<commit_message>
Saving some changes before refactoring
</commit_message>
<xml_diff>
--- a/data/clogging results.xlsx
+++ b/data/clogging results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casper/Semester 9/Master/Fullstack/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55620319-3C73-C849-8239-0A52FB20AEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985C9333-851C-1A48-AEFB-5A8BAD7CD03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{924581BB-33D1-DD46-A8CC-0A0848AB6A20}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="75">
   <si>
     <t>Name of file</t>
   </si>
@@ -170,9 +170,6 @@
     <t>15-03-LF.xlsx</t>
   </si>
   <si>
-    <t>SKIP FOR NOW</t>
-  </si>
-  <si>
     <t>Weird file setup</t>
   </si>
   <si>
@@ -197,9 +194,6 @@
     <t>From what i can see there is a spike at the beginning and a small spike at the end. Unclear what it is. Images to the right --&gt;</t>
   </si>
   <si>
-    <t>I think no clogging!</t>
-  </si>
-  <si>
     <t>01-10-xlsx</t>
   </si>
   <si>
@@ -221,9 +215,6 @@
     <t>Pressure was there for</t>
   </si>
   <si>
-    <t>Looks like 3-4 different runs, this is for the first crossing,</t>
-  </si>
-  <si>
     <t>7-12.xlsx</t>
   </si>
   <si>
@@ -252,6 +243,24 @@
   </si>
   <si>
     <t>Seems like there is a difference in data, my software does not controll it</t>
+  </si>
+  <si>
+    <t>There was 3  runs as i suspected, massiv, the graph did not showcase crossing. However the start of the data set seems to be a little weird.</t>
+  </si>
+  <si>
+    <t>can clearly see spikes</t>
+  </si>
+  <si>
+    <t>I think no clogging! Should remove the first part of the run in the files and see what happens</t>
+  </si>
+  <si>
+    <t>Looks like 3-4 different runs, this is for the first crossing, and after checking it was acutally 4 runs!!! Blockage in each of them respectively</t>
+  </si>
+  <si>
+    <t>Partial clogging</t>
+  </si>
+  <si>
+    <t>Dont understand the flow rate and descriptions</t>
   </si>
 </sst>
 </file>
@@ -261,10 +270,17 @@
   <numFmts count="1">
     <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -296,11 +312,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1089,9 +1106,10 @@
     <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="120" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.2">
@@ -1647,6 +1665,9 @@
       <c r="G16" s="1">
         <v>1.6863425925925928E-2</v>
       </c>
+      <c r="H16" t="s">
+        <v>10</v>
+      </c>
       <c r="I16" t="s">
         <v>13</v>
       </c>
@@ -1677,6 +1698,9 @@
       <c r="G17" s="1">
         <v>1.7175925925925924E-2</v>
       </c>
+      <c r="H17" t="s">
+        <v>10</v>
+      </c>
       <c r="I17" t="s">
         <v>13</v>
       </c>
@@ -1707,6 +1731,9 @@
       <c r="G18" s="1">
         <v>2.0833333333333333E-3</v>
       </c>
+      <c r="H18" t="s">
+        <v>70</v>
+      </c>
       <c r="I18" t="s">
         <v>11</v>
       </c>
@@ -1794,13 +1821,16 @@
       <c r="J21" t="s">
         <v>12</v>
       </c>
+      <c r="K21" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="C22">
         <v>3</v>
@@ -1820,6 +1850,9 @@
       <c r="A23" t="s">
         <v>43</v>
       </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
       <c r="C23">
         <v>5</v>
       </c>
@@ -1834,18 +1867,21 @@
         <v>12</v>
       </c>
       <c r="K23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>43</v>
       </c>
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
       <c r="C24">
         <v>3</v>
       </c>
       <c r="D24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F24" s="2" t="e">
         <f t="shared" si="1"/>
@@ -1862,6 +1898,9 @@
       <c r="A25" t="s">
         <v>43</v>
       </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
       <c r="C25">
         <v>5</v>
       </c>
@@ -1881,16 +1920,16 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26">
+        <v>3</v>
+      </c>
+      <c r="D26" t="s">
         <v>46</v>
-      </c>
-      <c r="B26" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26">
-        <v>3</v>
-      </c>
-      <c r="D26" t="s">
-        <v>47</v>
       </c>
       <c r="F26" s="2" t="e">
         <f t="shared" si="1"/>
@@ -1903,21 +1942,21 @@
         <v>12</v>
       </c>
       <c r="K26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C27">
         <v>5</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F27" s="2" t="e">
         <f t="shared" si="1"/>
@@ -1932,10 +1971,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C28">
         <v>3</v>
@@ -1956,10 +1995,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C29">
         <v>5</v>
@@ -1979,8 +2018,11 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>49</v>
+      <c r="A30" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
       </c>
       <c r="C30">
         <v>3</v>
@@ -1992,6 +2034,9 @@
       <c r="G30" s="1">
         <v>9.6064814814814819E-4</v>
       </c>
+      <c r="H30" t="s">
+        <v>26</v>
+      </c>
       <c r="I30" t="s">
         <v>11</v>
       </c>
@@ -2001,7 +2046,10 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="B31" t="s">
+        <v>9</v>
       </c>
       <c r="C31">
         <v>5</v>
@@ -2013,6 +2061,9 @@
       <c r="G31" s="1">
         <v>9.7222222222222219E-4</v>
       </c>
+      <c r="H31" t="s">
+        <v>26</v>
+      </c>
       <c r="I31" t="s">
         <v>11</v>
       </c>
@@ -2022,7 +2073,10 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="B32" t="s">
+        <v>9</v>
       </c>
       <c r="C32">
         <v>3</v>
@@ -2040,6 +2094,9 @@
       <c r="G32" s="1">
         <v>2.627314814814815E-3</v>
       </c>
+      <c r="H32" t="s">
+        <v>26</v>
+      </c>
       <c r="I32" t="s">
         <v>13</v>
       </c>
@@ -2047,12 +2104,15 @@
         <v>12</v>
       </c>
       <c r="K32" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
       </c>
       <c r="C33">
         <v>5</v>
@@ -2070,6 +2130,9 @@
       <c r="G33" s="1">
         <v>2.8472222222222223E-3</v>
       </c>
+      <c r="H33" t="s">
+        <v>26</v>
+      </c>
       <c r="I33" t="s">
         <v>13</v>
       </c>
@@ -2077,12 +2140,15 @@
         <v>12</v>
       </c>
       <c r="K33" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
       </c>
       <c r="C34">
         <v>3</v>
@@ -2100,6 +2166,9 @@
       <c r="G34" s="1">
         <v>1.2766203703703703E-2</v>
       </c>
+      <c r="H34" t="s">
+        <v>10</v>
+      </c>
       <c r="I34" t="s">
         <v>11</v>
       </c>
@@ -2109,7 +2178,10 @@
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
       </c>
       <c r="C35">
         <v>5</v>
@@ -2127,6 +2199,9 @@
       <c r="G35" s="1">
         <v>1.2789351851851852E-2</v>
       </c>
+      <c r="H35" t="s">
+        <v>10</v>
+      </c>
       <c r="I35" t="s">
         <v>11</v>
       </c>
@@ -2134,12 +2209,15 @@
         <v>12</v>
       </c>
       <c r="K35" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
       </c>
       <c r="C36">
         <v>3</v>
@@ -2157,6 +2235,9 @@
       <c r="G36" s="1">
         <v>1.275462962962963E-2</v>
       </c>
+      <c r="H36" t="s">
+        <v>10</v>
+      </c>
       <c r="I36" t="s">
         <v>13</v>
       </c>
@@ -2166,7 +2247,10 @@
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="B37" t="s">
+        <v>9</v>
       </c>
       <c r="C37">
         <v>5</v>
@@ -2184,6 +2268,9 @@
       <c r="G37" s="1">
         <v>1.2777777777777779E-2</v>
       </c>
+      <c r="H37" t="s">
+        <v>10</v>
+      </c>
       <c r="I37" t="s">
         <v>13</v>
       </c>
@@ -2191,12 +2278,15 @@
         <v>12</v>
       </c>
       <c r="K37" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
       </c>
       <c r="C38">
         <v>3</v>
@@ -2221,7 +2311,10 @@
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
       </c>
       <c r="C39">
         <v>5</v>
@@ -2243,12 +2336,15 @@
         <v>12</v>
       </c>
       <c r="K39" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="B40" t="s">
+        <v>9</v>
       </c>
       <c r="C40">
         <v>3</v>
@@ -2270,15 +2366,18 @@
         <v>12</v>
       </c>
       <c r="K40" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="S40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
       </c>
       <c r="C41">
         <v>5</v>
@@ -2300,12 +2399,15 @@
         <v>12</v>
       </c>
       <c r="K41" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="B42" t="s">
+        <v>23</v>
       </c>
       <c r="C42">
         <v>3</v>
@@ -2332,7 +2434,10 @@
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="B43" t="s">
+        <v>23</v>
       </c>
       <c r="C43">
         <v>5</v>
@@ -2359,7 +2464,10 @@
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="B44" t="s">
+        <v>23</v>
       </c>
       <c r="C44">
         <v>3</v>
@@ -2386,7 +2494,10 @@
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="B45" t="s">
+        <v>23</v>
       </c>
       <c r="C45">
         <v>5</v>
@@ -2411,12 +2522,15 @@
         <v>12</v>
       </c>
       <c r="K45" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
+      </c>
+      <c r="B46" t="s">
+        <v>9</v>
       </c>
       <c r="C46">
         <v>3</v>
@@ -2436,7 +2550,10 @@
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
+      </c>
+      <c r="B47" t="s">
+        <v>9</v>
       </c>
       <c r="C47">
         <v>5</v>
@@ -2454,12 +2571,15 @@
         <v>12</v>
       </c>
       <c r="K47" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
+      </c>
+      <c r="B48" t="s">
+        <v>9</v>
       </c>
       <c r="C48">
         <v>3</v>
@@ -2479,7 +2599,10 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
+      </c>
+      <c r="B49" t="s">
+        <v>9</v>
       </c>
       <c r="C49">
         <v>5</v>
@@ -2499,7 +2622,10 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="B50" t="s">
+        <v>23</v>
       </c>
       <c r="C50">
         <v>3</v>
@@ -2519,7 +2645,10 @@
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="B51" t="s">
+        <v>23</v>
       </c>
       <c r="C51">
         <v>5</v>
@@ -2539,7 +2668,10 @@
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="B52" t="s">
+        <v>23</v>
       </c>
       <c r="C52">
         <v>3</v>
@@ -2559,7 +2691,10 @@
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="B53" t="s">
+        <v>23</v>
       </c>
       <c r="C53">
         <v>5</v>
@@ -2577,12 +2712,15 @@
         <v>12</v>
       </c>
       <c r="K53" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
+      </c>
+      <c r="B54" t="s">
+        <v>9</v>
       </c>
       <c r="C54">
         <v>3</v>
@@ -2602,7 +2740,10 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
+      </c>
+      <c r="B55" t="s">
+        <v>9</v>
       </c>
       <c r="C55">
         <v>5</v>
@@ -2622,7 +2763,10 @@
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
+      </c>
+      <c r="B56" t="s">
+        <v>9</v>
       </c>
       <c r="C56">
         <v>3</v>
@@ -2642,7 +2786,10 @@
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
+      </c>
+      <c r="B57" t="s">
+        <v>9</v>
       </c>
       <c r="C57">
         <v>5</v>
@@ -2662,7 +2809,10 @@
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="B58" t="s">
+        <v>23</v>
       </c>
       <c r="C58">
         <v>3</v>
@@ -2679,10 +2829,16 @@
       <c r="J58" t="s">
         <v>12</v>
       </c>
+      <c r="K58" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="B59" t="s">
+        <v>23</v>
       </c>
       <c r="C59">
         <v>5</v>
@@ -2702,7 +2858,10 @@
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="B60" t="s">
+        <v>23</v>
       </c>
       <c r="C60">
         <v>3</v>
@@ -2722,7 +2881,10 @@
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="B61" t="s">
+        <v>23</v>
       </c>
       <c r="C61">
         <v>5</v>
@@ -2742,7 +2904,10 @@
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
+      </c>
+      <c r="B62" t="s">
+        <v>73</v>
       </c>
       <c r="C62">
         <v>3</v>
@@ -2756,7 +2921,10 @@
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
+      </c>
+      <c r="B63" t="s">
+        <v>73</v>
       </c>
       <c r="C63">
         <v>5</v>
@@ -2768,12 +2936,15 @@
         <v>12</v>
       </c>
       <c r="M63" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
+      </c>
+      <c r="B64" t="s">
+        <v>73</v>
       </c>
       <c r="C64">
         <v>3</v>
@@ -2787,7 +2958,10 @@
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
+      </c>
+      <c r="B65" t="s">
+        <v>73</v>
       </c>
       <c r="C65">
         <v>5</v>
@@ -2801,31 +2975,31 @@
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.2">
       <c r="S69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="107" spans="19:19" x14ac:dyDescent="0.2">
       <c r="S107" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="138" spans="19:19" x14ac:dyDescent="0.2">
       <c r="S138" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="175" spans="19:19" x14ac:dyDescent="0.2">
       <c r="S175" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="204" spans="19:19" x14ac:dyDescent="0.2">
       <c r="S204" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>